<commit_message>
sc: Check against reference also in testPivotTableFormatsGrandTotal
The testPivotTableFormatsGrandTotal still used checking specific
cells for background and font color, while most other tests use
checking against the reference that is contained in the document.
This changes the test and also modifies the document to put the
reference at the position that is expected and standard in other
test documents (one empty row between the pivot table end and
reference start).

Change-Id: Id309e998a8527e2cf1fe246917780cbd77beec5f
Reviewed-on: https://gerrit.collaboraoffice.com/c/online/+/2734
Reviewed-by: Miklos Vajna <vmiklos@collabora.com>
Tested-by: Jenkins CPCI <releng@collaboraoffice.com>
(cherry picked from commit 4b8061eedcf1944131fde98724ec0ee9d4b9709c)
Reviewed-on: https://gerrit.libreoffice.org/c/core/+/205788
Reviewed-by: Xisco Fauli <xiscofauli@libreoffice.org>
Tested-by: Jenkins
</commit_message>
<xml_diff>
--- a/sc/qa/unit/data/xlsx/pivot-table/PivotTableFormatsGrandTotal.xlsx
+++ b/sc/qa/unit/data/xlsx/pivot-table/PivotTableFormatsGrandTotal.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29917"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36FDE4DE-2793-4DD3-960E-1366CAD105F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8DA055D-B710-4FAF-977B-597C49C675E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="470" r:id="rId3"/>
+    <pivotCache cacheId="1567" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -464,7 +464,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76880066-9EFC-419F-8D56-7F109951BFC9}" name="PivotTable2" cacheId="470" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76880066-9EFC-419F-8D56-7F109951BFC9}" name="PivotTable2" cacheId="1567" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B3:G14" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
@@ -918,7 +918,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DB5B72E-F73B-4772-A355-5C5A98BEF845}">
-  <dimension ref="B3:G28"/>
+  <dimension ref="B3:G27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -1111,45 +1111,59 @@
         <v>26</v>
       </c>
     </row>
+    <row r="16" spans="2:7">
+      <c r="B16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="3"/>
+    </row>
     <row r="17" spans="2:7">
       <c r="B17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7">
+        <v>3</v>
+      </c>
+      <c r="F17" s="7">
+        <v>4</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" spans="2:7">
-      <c r="B18" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1</v>
-      </c>
-      <c r="E18" s="7">
-        <v>3</v>
-      </c>
-      <c r="F18" s="7">
-        <v>4</v>
-      </c>
-      <c r="G18" s="18" t="s">
-        <v>4</v>
+      <c r="B18" s="1">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <v>3</v>
+      </c>
+      <c r="D18" s="8">
+        <v>6</v>
+      </c>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="19">
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="2:7">
-      <c r="B19" s="1">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1">
-        <v>3</v>
-      </c>
+      <c r="B19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2"/>
       <c r="D19" s="8">
         <v>6</v>
       </c>
@@ -1160,102 +1174,102 @@
       </c>
     </row>
     <row r="20" spans="2:7">
-      <c r="B20" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20" s="2"/>
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
       <c r="D20" s="8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="19">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="2:7">
-      <c r="B21" s="1">
+      <c r="B21" s="4"/>
+      <c r="C21" s="11">
         <v>2</v>
       </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" s="8">
-        <v>8</v>
-      </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="19">
-        <v>8</v>
+      <c r="D21" s="12">
+        <v>1</v>
+      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="20">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:7">
       <c r="B22" s="4"/>
       <c r="C22" s="11">
-        <v>2</v>
-      </c>
-      <c r="D22" s="12">
-        <v>1</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D22" s="12"/>
       <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="20">
-        <v>1</v>
+      <c r="F22" s="5">
+        <v>3</v>
+      </c>
+      <c r="G22" s="13">
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="2:7">
       <c r="B23" s="4"/>
       <c r="C23" s="11">
+        <v>7</v>
+      </c>
+      <c r="D23" s="12"/>
+      <c r="E23" s="5">
+        <v>5</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7">
+      <c r="B24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5">
-        <v>3</v>
-      </c>
-      <c r="G23" s="13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7">
-      <c r="B24" s="4"/>
-      <c r="C24" s="11">
+      <c r="C24" s="2"/>
+      <c r="D24" s="8">
+        <v>9</v>
+      </c>
+      <c r="E24" s="9">
+        <v>5</v>
+      </c>
+      <c r="F24" s="9">
+        <v>3</v>
+      </c>
+      <c r="G24" s="10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7">
+      <c r="B25" s="1">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1">
+        <v>9</v>
+      </c>
+      <c r="D25" s="8"/>
+      <c r="E25" s="9">
+        <v>3</v>
+      </c>
+      <c r="F25" s="9"/>
+      <c r="G25" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7">
+      <c r="B26" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="5">
-        <v>5</v>
-      </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="13">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7">
-      <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="8">
-        <v>9</v>
-      </c>
-      <c r="E25" s="9">
-        <v>5</v>
-      </c>
-      <c r="F25" s="9">
-        <v>3</v>
-      </c>
-      <c r="G25" s="10">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7">
-      <c r="B26" s="1">
-        <v>3</v>
-      </c>
-      <c r="C26" s="1">
-        <v>9</v>
-      </c>
+      <c r="C26" s="2"/>
       <c r="D26" s="8"/>
       <c r="E26" s="9">
         <v>3</v>
@@ -1266,34 +1280,20 @@
       </c>
     </row>
     <row r="27" spans="2:7">
-      <c r="B27" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="9">
-        <v>3</v>
-      </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7">
-      <c r="B28" s="16" t="s">
+      <c r="B27" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="14">
+      <c r="C27" s="17"/>
+      <c r="D27" s="14">
         <v>15</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E27" s="22">
         <v>8</v>
       </c>
-      <c r="F28" s="15">
-        <v>3</v>
-      </c>
-      <c r="G28" s="21">
+      <c r="F27" s="15">
+        <v>3</v>
+      </c>
+      <c r="G27" s="21">
         <v>26</v>
       </c>
     </row>

</xml_diff>